<commit_message>
.env configuration and config class
</commit_message>
<xml_diff>
--- a/weather_data.xlsx
+++ b/weather_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -650,6 +650,102 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lisbon</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D8" t="n">
+        <v>22.21</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-04-13 18:00:36</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>69</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1021</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>broken clouds</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lisbon</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" t="n">
+        <v>15</v>
+      </c>
+      <c r="D9" t="n">
+        <v>22.21</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-04-13 18:00:42</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>69</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>broken clouds</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lisbon</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D10" t="n">
+        <v>22.21</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-04-13 18:00:47</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>69</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1021</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>broken clouds</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
save to mysql function
</commit_message>
<xml_diff>
--- a/weather_data.xlsx
+++ b/weather_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -746,6 +746,102 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Lisbon</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>25</v>
+      </c>
+      <c r="C11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D11" t="n">
+        <v>14.83</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-04-20 18:12:15</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1010</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>clear sky</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Lisbon</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>25</v>
+      </c>
+      <c r="C12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D12" t="n">
+        <v>14.83</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-04-20 18:12:20</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>30</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1010</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>clear sky</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lisbon</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>25</v>
+      </c>
+      <c r="C13" t="n">
+        <v>25</v>
+      </c>
+      <c r="D13" t="n">
+        <v>14.83</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-04-20 18:12:26</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>30</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1010</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>clear sky</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>